<commit_message>
Dodanie testów i aktualizacja main'a
</commit_message>
<xml_diff>
--- a/raport_koncowy.xlsx
+++ b/raport_koncowy.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Szczegóły_Rozliczeń" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Podsumowanie_Działów" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Szczegóły" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +28,23 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000070C0"/>
+        <bgColor rgb="000070C0"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -56,9 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -430,37 +442,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ID_Pracownika</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Imie</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Nazwisko</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Dzial</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Stawka_Godzinowa</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Przepracowane_Godziny</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Wynagrodzenie_Calkowite</t>
         </is>
@@ -608,89 +620,6 @@
         <v>82</v>
       </c>
       <c r="G6" t="n">
-        <v>16400</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Dzial</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Przepracowane_Godziny</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Wynagrodzenie_Calkowite</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>HR</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>75</v>
-      </c>
-      <c r="C2" t="n">
-        <v>5250</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>IT</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>125</v>
-      </c>
-      <c r="C3" t="n">
-        <v>14600</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sprzedaż</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>80</v>
-      </c>
-      <c r="C4" t="n">
-        <v>6800</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Zarząd</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>82</v>
-      </c>
-      <c r="C5" t="n">
         <v>16400</v>
       </c>
     </row>

</xml_diff>